<commit_message>
Sincroniza el sitio con el modelo del 20-10-2026
Estadísticas, tabla de cantidades (nuevos nombres de tipos, 4 faldones de cubierta,
aparatos sanitarios, mobiliario y emplazamiento), 16 proveedores, Tabla NDI v9,
PEB/EETT/Parámetros actualizados, lámina A101 e IFC4x3 re-exportados, visor 3D con
materiales y categorías nuevas, zip y presentación PDF regenerados.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
+++ b/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\AppData\Local\Temp\claude\C--Users-user-OneDrive-Escritorio-CURSO-BIM-IA-Claude\63969694-b2af-4bd1-919d-9b63abdf2687\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\AppData\Local\Temp\claude\C--Users-user-OneDrive-Escritorio-CURSO-BIM-IA-Claude\c32490e3-48b8-4c11-9b04-e055733501a8\scratchpad\audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17A66600-7C05-4CE1-8877-71D13124F913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5A97AB-B1C1-4E9D-9C4F-EA5B8E171ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proveedores" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="135">
   <si>
     <t>Categoría</t>
   </si>
@@ -77,9 +77,6 @@
     <t>Cubierta</t>
   </si>
   <si>
-    <t>CUBIERTA_ZINC_ONDULADO_MADERA</t>
-  </si>
-  <si>
     <t>Cubiertas Nacionales</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>https://www.melon.cl/wp-content/uploads/2023/03/Ficha-Hormigon-con-Fibra_CC.pdf</t>
   </si>
   <si>
-    <t>RADIER_PULIDO_INT_HA_2cm</t>
-  </si>
-  <si>
     <t>Sika Chile</t>
   </si>
   <si>
@@ -176,9 +170,6 @@
     <t>Armazón estructural</t>
   </si>
   <si>
-    <t>VIGA_Pino Radiata Dimensionada_Rectangular</t>
-  </si>
-  <si>
     <t>Arauco — MSD</t>
   </si>
   <si>
@@ -197,9 +188,6 @@
     <t>Muro cortina — montante</t>
   </si>
   <si>
-    <t>MADERA_1.25X10cm</t>
-  </si>
-  <si>
     <t>Pino Radiata Cepillado</t>
   </si>
   <si>
@@ -221,9 +209,6 @@
     <t>Puerta</t>
   </si>
   <si>
-    <t>PRT_INT_SIMPLE_MADERA</t>
-  </si>
-  <si>
     <t>Moldupanel (Puertas Chile)</t>
   </si>
   <si>
@@ -248,9 +233,6 @@
     <t>Puerta — herrajes</t>
   </si>
   <si>
-    <t>PRT_INT_SIMPLE_MADERA (bisagras/cerradura)</t>
-  </si>
-  <si>
     <t>Häfele (vía El Carpintero, distribuidor)</t>
   </si>
   <si>
@@ -275,9 +257,6 @@
     <t>Sanitarios</t>
   </si>
   <si>
-    <t>SAN_INT_WC_VALENCIA_MURO / SAN_INT_LAVAMANOS_CIRO</t>
-  </si>
-  <si>
     <t>Fanaloza</t>
   </si>
   <si>
@@ -332,9 +311,6 @@
     <t>Los 8 primeros ya están referenciados como Fabricante/Modelo/URL directamente en los tipos y materiales del modelo Revit (HAB_ARQ_MODELO_R01.rvt).</t>
   </si>
   <si>
-    <t>Häfele, Protierra y Sodimac/Construmart se agregan para cerrar categorías sin proveedor confirmado (herrajes, sistema constructivo de quincha, y punto de abastecimiento local).</t>
-  </si>
-  <si>
     <t>Verificación en vivo (navegador, 09-09-2026): Cubiertas Nacionales, Melón, Sika, Arauco, Fanaloza, Puertas Chile/Moldupanel, Häfele/El Carpintero y Protierra confirmados activos; datos de contacto de Moldupanel y Häfele actualizados con la información real encontrada en sus sitios.</t>
   </si>
   <si>
@@ -347,10 +323,109 @@
     <t>Suelo / Cimentación</t>
   </si>
   <si>
-    <t>RADIER_INT_HA_15cm / ZAPATA_Hormigon Armado_Aislada (ficha Melón como referencia)</t>
-  </si>
-  <si>
-    <t>Fecha: 09-09-2026 (actualizado 02-10-2026: panel de muro cortina = Empty; zapatas referenciadas a la ficha Melón)</t>
+    <t>CUBIERTA_ZINC ONDULADO_10cm</t>
+  </si>
+  <si>
+    <t>RADIER_INT_HA_15cm / FUNDACIÓN AISLADA_HA_60x60x50cm (ficha Melón como referencia)</t>
+  </si>
+  <si>
+    <t>PAV_INT_HORMIGON PULIDO_2cm</t>
+  </si>
+  <si>
+    <t>VIGA_PINO RADIATA_Rectangular</t>
+  </si>
+  <si>
+    <t>12.5x100mm_PINO RADIATA</t>
+  </si>
+  <si>
+    <t>PRT_Puerta_INT_Simple_1 Panel_PINO RADIATA</t>
+  </si>
+  <si>
+    <t>PRT_Puerta_INT_Simple_1 Panel_PINO RADIATA (bisagras/cerradura)</t>
+  </si>
+  <si>
+    <t>PLM_WC_ceramica_New Valencia a muro / PLM_Lavamanos_ceramica_Ciro pedestal</t>
+  </si>
+  <si>
+    <t>Aparatos sanitarios</t>
+  </si>
+  <si>
+    <t>PLM_Bebedero_acero inoxidable_Wolfen sensor pie</t>
+  </si>
+  <si>
+    <t>Reece Australia Pty Ltd</t>
+  </si>
+  <si>
+    <t>Wolfen Sensor Drinking Fountain WDF2SS (cód. 1308142)</t>
+  </si>
+  <si>
+    <t>118 Burwood Hwy, Burwood VIC 3125, Australia</t>
+  </si>
+  <si>
+    <t>+61 3 9274 0000</t>
+  </si>
+  <si>
+    <t>admin@reece.com.au</t>
+  </si>
+  <si>
+    <t>reece.com.au</t>
+  </si>
+  <si>
+    <t>https://digitalassets.reecegroup.com.au/m/47a8b771eca7c04f/original/Specification-Sheet-Wolfen-Drinking-Fountain.pdf</t>
+  </si>
+  <si>
+    <t>Emplazamiento — bicicletero</t>
+  </si>
+  <si>
+    <t>SITIO_Bicicletero_acero galvanizado_U</t>
+  </si>
+  <si>
+    <t>Dero Bike Racks</t>
+  </si>
+  <si>
+    <t>U-Lockit (cód. G2040500)</t>
+  </si>
+  <si>
+    <t>dero.com</t>
+  </si>
+  <si>
+    <t>http://www.dero.com/product/u-lockit/</t>
+  </si>
+  <si>
+    <t>Emplazamiento — banca</t>
+  </si>
+  <si>
+    <t>SITIO_Banca_acero galvanizado y madera</t>
+  </si>
+  <si>
+    <t>Metalco</t>
+  </si>
+  <si>
+    <t>Big Harris (ficha de terceros; sin ficha oficial obtenida)</t>
+  </si>
+  <si>
+    <t>metalco.it</t>
+  </si>
+  <si>
+    <t>https://www.archiexpo.com/prod/metalco/product-56172-338958.html</t>
+  </si>
+  <si>
+    <t>Mobiliario — lavaplatos</t>
+  </si>
+  <si>
+    <t>MBL_Mueble base cocina_Lavaplatos</t>
+  </si>
+  <si>
+    <t>Lavaplatos de sobreponer con escurridor 80x50x14,5 cm, cód. JHSM2614DE11CF / JHSM2614IZ11CF (referencia propuesta)</t>
+  </si>
+  <si>
+    <t>https://www.fanaloza.cl/wp-content/uploads/2024/11/Catalogo-Ferretero_2025.pdf</t>
+  </si>
+  <si>
+    <t>Fecha: 09-09-2026 (actualizado 02-10-2026: panel de muro cortina = Empty; zapatas referenciadas a la ficha Melón) · actualizado 20-10-2026: nombres según el protocolo DIPBIM; se agregan Reece, Dero, Metalco y lavaplatos Fanaloza</t>
+  </si>
+  <si>
+    <t>Häfele, Protierra y Sodimac/Construmart cierran categorías sin proveedor confirmado (herrajes, sistema constructivo de quincha y punto de abastecimiento local). Reece, Dero y Metalco corresponden a los objetos BIM de bebedero, bicicletero y banca; Reece es un producto australiano usado como referencia (equivalente local por definir) y de Metalco solo hay fichas de terceros.</t>
   </si>
 </sst>
 </file>
@@ -747,7 +822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -789,7 +864,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -818,322 +893,438 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>14</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H5" s="3" t="s">
+    </row>
+    <row r="6" spans="1:9" ht="51" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="B7" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="E7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="B8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="E8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="51" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="I11" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="3" t="s">
+    </row>
+    <row r="12" spans="1:9" ht="51" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="B12" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:9" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="E17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="F17" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="G17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="I13" s="3" t="s">
+      <c r="I17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1152,17 +1343,17 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
@@ -1170,22 +1361,22 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Proveedores: sanitarios, lavamanos y lavaplatos en un solo punto (web y Excel)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
+++ b/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b91da64fcc1594/Escritorio/CURSO BIM^MIA/Claude/Pausa_Maule/03_Documentos_Tecnicos/Proveedores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D053D23-7FE2-4CD3-BE16-38E7C7F886D0}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B755677A-0719-467A-AFDF-A7D674D8CE22}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="1935" windowWidth="28170" windowHeight="14985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proveedores" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="149">
   <si>
     <t>Categoría</t>
   </si>
@@ -343,15 +343,9 @@
     <t>Sanitarios</t>
   </si>
   <si>
-    <t>41x69cm (inodoro New Valencia a muro) / 53x41cm (lavamanos Ciro pedestal)</t>
-  </si>
-  <si>
     <t>Fanaloza</t>
   </si>
   <si>
-    <t>New Valencia a Muro / Lavamanos Ciro</t>
-  </si>
-  <si>
     <t>Av. Eduardo Frei Montalva km 19,5, Colina, RM</t>
   </si>
   <si>
@@ -364,12 +358,6 @@
     <t>fanaloza.cl</t>
   </si>
   <si>
-    <t>https://www.fanaloza.cl/producto/inodoro-new-valencia-a-muro/</t>
-  </si>
-  <si>
-    <t>10.01.01 / 10.01.02</t>
-  </si>
-  <si>
     <t>Aparatos sanitarios</t>
   </si>
   <si>
@@ -439,21 +427,6 @@
     <t>11.01.01</t>
   </si>
   <si>
-    <t>Mobiliario — lavaplatos</t>
-  </si>
-  <si>
-    <t>80x60cm (mueble base lavaplatos)</t>
-  </si>
-  <si>
-    <t>Lavaplatos de sobreponer con escurridor 80x50x14,5 cm, cód. JHSM2614DE11CF / JHSM2614IZ11CF (referencia propuesta)</t>
-  </si>
-  <si>
-    <t>https://www.fanaloza.cl/wp-content/uploads/2024/11/Catalogo-Ferretero_2025.pdf</t>
-  </si>
-  <si>
-    <t>10.01.03</t>
-  </si>
-  <si>
     <t>Punto de venta local</t>
   </si>
   <si>
@@ -482,6 +455,20 @@
   </si>
   <si>
     <t>https://857f7855-aec8-45b4-bf05-510e3fd4d166.usrfiles.com/ugd/857f78_8bf690ef7ef54d6d9bec6e0aa665dedf.pdf</t>
+  </si>
+  <si>
+    <t>41x69cm (inodoro New Valencia a muro) / 53x41cm (lavamanos Ciro pedestal) / 80x60cm (mueble base lavaplatos)</t>
+  </si>
+  <si>
+    <t>Inodoro New Valencia a Muro / Lavamanos Ciro con pedestal / Lavaplatos de sobreponer con escurridor 80x50x14,5 cm, cód. JHSM2614DE11CF / JHSM2614IZ11CF (referencia propuesta)</t>
+  </si>
+  <si>
+    <t>https://www.fanaloza.cl/producto/inodoro-new-valencia-a-muro/
+https://www.fanaloza.cl/producto/lavamanos-ciro-con-pedestal/
+https://www.fanaloza.cl/wp-content/uploads/2024/11/Catalogo-Ferretero_2025.pdf</t>
+  </si>
+  <si>
+    <t>10.01.01 / 10.01.02 / 10.01.03</t>
   </si>
 </sst>
 </file>
@@ -867,7 +854,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1265,53 +1252,53 @@
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>106</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="I13" s="2" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>15</v>
@@ -1320,141 +1307,109 @@
         <v>15</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="I15" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D16" s="2" t="s">
+    </row>
+    <row r="17" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="E17" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="F17" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="G17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="I17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" s="3" t="s">
         <v>142</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Proveedores: bebedero dentro del punto de sanitarios (web y Excel)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
+++ b/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b91da64fcc1594/Escritorio/CURSO BIM^MIA/Claude/Pausa_Maule/03_Documentos_Tecnicos/Proveedores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B755677A-0719-467A-AFDF-A7D674D8CE22}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B6039F3-9EEE-4457-8406-66A128B1B263}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="4680" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="141">
   <si>
     <t>Categoría</t>
   </si>
@@ -343,9 +343,6 @@
     <t>Sanitarios</t>
   </si>
   <si>
-    <t>Fanaloza</t>
-  </si>
-  <si>
     <t>Av. Eduardo Frei Montalva km 19,5, Colina, RM</t>
   </si>
   <si>
@@ -355,30 +352,6 @@
     <t>ventas@fanaloza.cl</t>
   </si>
   <si>
-    <t>fanaloza.cl</t>
-  </si>
-  <si>
-    <t>Aparatos sanitarios</t>
-  </si>
-  <si>
-    <t>BAG-40_32x32x112cm</t>
-  </si>
-  <si>
-    <t>FAMAVA</t>
-  </si>
-  <si>
-    <t>Bebedero de agua BAG-40 (acero inoxidable, 320x320x1120 mm)</t>
-  </si>
-  <si>
-    <t>Chile (fabricante nacional)</t>
-  </si>
-  <si>
-    <t>famava.cl</t>
-  </si>
-  <si>
-    <t>10.01.04</t>
-  </si>
-  <si>
     <t>Emplazamiento — bicicletero</t>
   </si>
   <si>
@@ -451,24 +424,29 @@
     <t>—</t>
   </si>
   <si>
-    <t>https://www.famava.cl/CatalogoPDF/9/BAG-40/</t>
-  </si>
-  <si>
     <t>https://857f7855-aec8-45b4-bf05-510e3fd4d166.usrfiles.com/ugd/857f78_8bf690ef7ef54d6d9bec6e0aa665dedf.pdf</t>
   </si>
   <si>
-    <t>41x69cm (inodoro New Valencia a muro) / 53x41cm (lavamanos Ciro pedestal) / 80x60cm (mueble base lavaplatos)</t>
-  </si>
-  <si>
-    <t>Inodoro New Valencia a Muro / Lavamanos Ciro con pedestal / Lavaplatos de sobreponer con escurridor 80x50x14,5 cm, cód. JHSM2614DE11CF / JHSM2614IZ11CF (referencia propuesta)</t>
+    <t>41x69cm (inodoro New Valencia a muro) / 53x41cm (lavamanos Ciro pedestal) / 80x60cm (mueble base lavaplatos) / BAG-40_32x32x112cm (bebedero)</t>
+  </si>
+  <si>
+    <t>Fanaloza (inodoro, lavamanos, lavaplatos) / FAMAVA (bebedero)</t>
+  </si>
+  <si>
+    <t>Inodoro New Valencia a Muro / Lavamanos Ciro con pedestal / Lavaplatos de sobreponer con escurridor 80x50x14,5 cm, cód. JHSM2614DE11CF / JHSM2614IZ11CF (referencia propuesta) / Bebedero de agua BAG-40 (acero inoxidable, 320x320x1120 mm)</t>
+  </si>
+  <si>
+    <t>fanaloza.cl
+famava.cl</t>
   </si>
   <si>
     <t>https://www.fanaloza.cl/producto/inodoro-new-valencia-a-muro/
 https://www.fanaloza.cl/producto/lavamanos-ciro-con-pedestal/
-https://www.fanaloza.cl/wp-content/uploads/2024/11/Catalogo-Ferretero_2025.pdf</t>
-  </si>
-  <si>
-    <t>10.01.01 / 10.01.02 / 10.01.03</t>
+https://www.fanaloza.cl/wp-content/uploads/2024/11/Catalogo-Ferretero_2025.pdf
+https://www.famava.cl/CatalogoPDF/9/BAG-40/</t>
+  </si>
+  <si>
+    <t>10.01.01 / 10.01.02 / 10.01.03 / 10.01.04</t>
   </si>
 </sst>
 </file>
@@ -567,6 +545,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -854,7 +836,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1252,71 +1234,71 @@
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>106</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="H13" s="2" t="s">
-        <v>111</v>
+        <v>138</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>117</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>119</v>
       </c>
@@ -1333,83 +1315,51 @@
         <v>123</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="H15" s="2" t="s">
+    </row>
+    <row r="16" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="J15" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="F16" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="G16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>133</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Proveedores: banca como mobiliario
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
+++ b/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b91da64fcc1594/Escritorio/CURSO BIM^MIA/Claude/Pausa_Maule/03_Documentos_Tecnicos/Proveedores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B6039F3-9EEE-4457-8406-66A128B1B263}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{673E1308-BB6E-4095-8079-AACAEEBEAD4D}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="4680" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -379,9 +379,6 @@
     <t>11.01.02</t>
   </si>
   <si>
-    <t>Emplazamiento — banca</t>
-  </si>
-  <si>
     <t>INSITU_250x40x45cm</t>
   </si>
   <si>
@@ -447,6 +444,9 @@
   </si>
   <si>
     <t>10.01.01 / 10.01.02 / 10.01.03 / 10.01.04</t>
+  </si>
+  <si>
+    <t>Mobiliario — banca</t>
   </si>
 </sst>
 </file>
@@ -1239,13 +1239,13 @@
         <v>106</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>107</v>
@@ -1257,13 +1257,13 @@
         <v>109</v>
       </c>
       <c r="H13" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1292,7 +1292,7 @@
         <v>117</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>118</v>
@@ -1300,66 +1300,66 @@
     </row>
     <row r="15" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Proveedores: elementos de sanitarios (lavaplatos, lavamanos, WC, bebedero) con su ficha
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
+++ b/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b91da64fcc1594/Escritorio/CURSO BIM^MIA/Claude/Pausa_Maule/03_Documentos_Tecnicos/Proveedores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{673E1308-BB6E-4095-8079-AACAEEBEAD4D}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_55A7F2FC55098790D499234AD3675D69D9F8956B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DDE4AB7-50A8-4E8D-A46B-042FD4478D39}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="4680" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -424,29 +424,43 @@
     <t>https://857f7855-aec8-45b4-bf05-510e3fd4d166.usrfiles.com/ugd/857f78_8bf690ef7ef54d6d9bec6e0aa665dedf.pdf</t>
   </si>
   <si>
-    <t>41x69cm (inodoro New Valencia a muro) / 53x41cm (lavamanos Ciro pedestal) / 80x60cm (mueble base lavaplatos) / BAG-40_32x32x112cm (bebedero)</t>
-  </si>
-  <si>
-    <t>Fanaloza (inodoro, lavamanos, lavaplatos) / FAMAVA (bebedero)</t>
-  </si>
-  <si>
-    <t>Inodoro New Valencia a Muro / Lavamanos Ciro con pedestal / Lavaplatos de sobreponer con escurridor 80x50x14,5 cm, cód. JHSM2614DE11CF / JHSM2614IZ11CF (referencia propuesta) / Bebedero de agua BAG-40 (acero inoxidable, 320x320x1120 mm)</t>
+    <t>Mobiliario — banca</t>
+  </si>
+  <si>
+    <t>Lavaplatos (80x60cm, mueble base)
+Lavamanos (53x41cm, Ciro pedestal)
+WC (41x69cm, New Valencia a muro)
+Bebedero (BAG-40_32x32x112cm)</t>
+  </si>
+  <si>
+    <t>Fanaloza
+Fanaloza
+Fanaloza
+FAMAVA</t>
+  </si>
+  <si>
+    <t>Lavaplatos de sobreponer con escurridor 80x50x14,5 cm, cód. JHSM2614DE11CF / JHSM2614IZ11CF (referencia propuesta)
+Lavamanos Ciro con pedestal
+Inodoro New Valencia a muro
+Bebedero de agua BAG-40 (acero inoxidable, 320x320x1120 mm)</t>
   </si>
   <si>
     <t>fanaloza.cl
+fanaloza.cl
+fanaloza.cl
 famava.cl</t>
   </si>
   <si>
-    <t>https://www.fanaloza.cl/producto/inodoro-new-valencia-a-muro/
+    <t>https://www.fanaloza.cl/wp-content/uploads/2024/11/Catalogo-Ferretero_2025.pdf
 https://www.fanaloza.cl/producto/lavamanos-ciro-con-pedestal/
-https://www.fanaloza.cl/wp-content/uploads/2024/11/Catalogo-Ferretero_2025.pdf
+https://www.fanaloza.cl/producto/inodoro-new-valencia-a-muro/
 https://www.famava.cl/CatalogoPDF/9/BAG-40/</t>
   </si>
   <si>
-    <t>10.01.01 / 10.01.02 / 10.01.03 / 10.01.04</t>
-  </si>
-  <si>
-    <t>Mobiliario — banca</t>
+    <t>10.01.03
+10.01.02
+10.01.01
+10.01.04</t>
   </si>
 </sst>
 </file>
@@ -1239,13 +1253,13 @@
         <v>106</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>107</v>
@@ -1257,13 +1271,13 @@
         <v>109</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1300,7 +1314,7 @@
     </row>
     <row r="15" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>119</v>

</xml_diff>